<commit_message>
Update content-calendar.xlsx after carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -819,7 +819,32 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>The Brilliant Jerk Problem, Recognise the Real Cost, Diagnose Before You Act, Intervene With Structure, Reinforce Culture, 6 Mistakes, 30-Day Action Plan</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>8,8,8,8,8,8,8</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>7 carousels from blog post. YouTube hit daily limit. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after carousel run 2026-03-25
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -987,7 +987,32 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>decision-fatigue-intro, decision-architecture, meeting-design, energy-management, cognitive-load-reduction, team-structure-decisions, decision-fatigue-mistakes</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>8, 8, 7, 8, 7, 8, 8</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X, Google Business, Bluesky (5/7 carousels scheduled; 2 pending rate limit)</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>TikTok/YouTube at daily limits; Pinterest no boards; Carousels 6-7 hit Buffer rate limit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after Steps After Working Genius carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1071,7 +1071,32 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Your First Week After Working Genius, Month One: Build the Foundation, Redesign How Your Team Works, Make Working Genius Stick, Build a Working Genius Culture</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>7, 8, 8, 8, 7</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>5 carousels, 45 posts scheduled across 9 platforms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after WG-Hiring carousel run 2026-03-25
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1113,7 +1113,32 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>wg-hiring-foundation, wg-hiring-diagnosis, wg-hiring-job-descriptions, wg-hiring-interviews, wg-hiring-assessment, wg-hiring-decisions, wg-hiring-onboarding, wg-hiring-mistakes, wg-hiring-advanced, wg-hiring-measuring</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>7x10 (70 total)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube, TikTok (90 posts)</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>10 carousels, 10 videos, 10 pins. YouTube Mar 26-27, TikTok Mar 29.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after sleep-leadership carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1155,7 +1155,32 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>sleep-leadership-stats, sleep-protect-your-window, sleep-manage-your-inputs, sleep-environment-and-light, sleep-stress-and-rumination, sleep-culture-and-recovery, sleep-mistakes-leaders-make</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>8, 6, 6, 8, 6, 8, 7</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, YouTube (6/7 Mar 30, 1/7 Mar 31)</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>7 carousels from blog post. TikTok hit daily limit. Pinterest no boards. YouTube carousel 7 scheduled Mar 31 (Mar 30 full).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after loneliness carousel run 2026-03-25
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1197,7 +1197,32 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>loneliness-external-support, loneliness-honest-culture, loneliness-unique-pressures, loneliness-personal-wellbeing, loneliness-daily-habits, loneliness-mistakes, loneliness-30-day-plan</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>7, 7, 7, 7, 7, 7, 7</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, YouTube, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>63 posts across 9 platforms. Pinterest skipped. YouTube Apr 6-10. TikTok Apr 5-6.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Expand content calendar with 140 items: testimonials, services, pain points, frameworks, BTS, stats
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1232,14 +1232,11 @@
           <t>Caring Hurts: The Hidden Cost of Leadership</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/caring-hurts-leadership</t>
-        </is>
-      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Blog Post</t>
+          <t>Blog</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1254,14 +1251,11 @@
           <t>Book Rec: Leaders Eat Last by Simon Sinek</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>https://www.simonandschuster.com/books/Leaders-Eat-Last/Simon-Sinek/9781591845324</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Book Recommendation</t>
+          <t>Book Rec</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1273,17 +1267,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Podcast Rec: Craig Groeschel Leadership Podcast</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>https://www.life.church/leadershippodcast/</t>
-        </is>
-      </c>
+          <t>My Team Nods But Nothing Changes</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Podcast Recommendation</t>
+          <t>Pain Point</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1295,17 +1286,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Imposter Syndrome as a Leader</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/imposter-syndrome-leader</t>
-        </is>
-      </c>
+          <t>Podcast Rec: Craig Groeschel Leadership Podcast</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Blog Post</t>
+          <t>Podcast Rec</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1317,17 +1305,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Book Rec: Unreasonable Hospitality by Will Guidara</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>https://www.unreasonablehospitality.com/</t>
-        </is>
-      </c>
+          <t>Testimonial: Kathy Dickson, CEO ASBA</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Book Recommendation</t>
+          <t>Testimonial</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1339,17 +1324,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Podcast Rec: HBR IdeaCast</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>https://hbr.org/2018/01/podcast-ideacast</t>
-        </is>
-      </c>
+          <t>Service: Leadership Team Offsite for Corporates</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Podcast Recommendation</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1361,17 +1343,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Leading Through Uncertainty</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/leading-through-uncertainty</t>
-        </is>
-      </c>
+          <t>The 5 Dysfunctions of a Team Explained</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Blog Post</t>
+          <t>Framework</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1383,17 +1362,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Book Rec: Radical Candor by Kim Scott</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>https://www.radicalcandor.com/the-book/</t>
-        </is>
-      </c>
+          <t>Imposter Syndrome as a Leader</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Book Recommendation</t>
+          <t>Blog</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1405,17 +1381,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Podcast Rec: WorkLife with Adam Grant</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>https://adamgrant.net/podcasts/worklife/</t>
-        </is>
-      </c>
+          <t>Book Rec: Unreasonable Hospitality by Will Guidara</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Podcast Recommendation</t>
+          <t>Book Rec</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1427,17 +1400,14 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Signs Your Executive Team is Dysfunctional</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/signs-executive-team-dysfunctional</t>
-        </is>
-      </c>
+          <t>We Keep Losing Good Teachers</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Blog Post</t>
+          <t>Pain Point</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1449,17 +1419,14 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Book Rec: Extreme Ownership by Jocko Willink</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>https://echelonfront.com/extreme-ownership/</t>
-        </is>
-      </c>
+          <t>Podcast Rec: HBR IdeaCast</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Book Recommendation</t>
+          <t>Podcast Rec</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1471,17 +1438,14 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Podcast Rec: The Learning Leader Show with Ryan Hawk</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>https://learningleader.com/</t>
-        </is>
-      </c>
+          <t>Testimonial: Michael Quach, Redlands College</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Podcast Recommendation</t>
+          <t>Testimonial</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1493,17 +1457,14 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>The Five Dysfunctions of a Team (Summary)</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/five-dysfunctions-summary</t>
-        </is>
-      </c>
+          <t>Service: Working Genius Workshop for Schools</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Blog Post</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1515,17 +1476,14 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Book Rec: Crucial Conversations by Patterson et al</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>https://cruciallearning.com/crucial-conversations-book/</t>
-        </is>
-      </c>
+          <t>What Actually Happens in a Working Genius Session</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Book Recommendation</t>
+          <t>Behind the Scenes</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1537,17 +1495,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Podcast Rec: Dare to Lead with Brene Brown</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>https://brenebrown.com/podcast/dare-to-lead/</t>
-        </is>
-      </c>
+          <t>Leading Through Uncertainty</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Podcast Recommendation</t>
+          <t>Blog</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1559,17 +1514,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Vulnerability-Based Trust</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/vulnerability-based-trust</t>
-        </is>
-      </c>
+          <t>Book Rec: Radical Candor by Kim Scott</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Blog Post</t>
+          <t>Book Rec</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1581,17 +1533,14 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Book Rec: Atomic Habits by James Clear</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>https://jamesclear.com/atomic-habits</t>
-        </is>
-      </c>
+          <t>Every Year We Set Priorities and Do the Same Things</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Book Recommendation</t>
+          <t>Pain Point</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1603,17 +1552,14 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Podcast Rec: The John Maxwell Leadership Podcast</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>https://johnmaxwell.com/podcast/</t>
-        </is>
-      </c>
+          <t>Podcast Rec: WorkLife with Adam Grant</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Podcast Recommendation</t>
+          <t>Podcast Rec</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1625,17 +1571,14 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Tips for Your First Year as Principal</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/tips-first-year-principal</t>
-        </is>
-      </c>
+          <t>Testimonial: Brett Bleakley, Livingstone Christian School</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Blog Post</t>
+          <t>Testimonial</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1647,17 +1590,14 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Book Rec: Hidden Potential by Adam Grant</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>https://adamgrant.net/book/hidden-potential/</t>
-        </is>
-      </c>
+          <t>Service: Keynote Speaking for Conferences</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Book Recommendation</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1669,17 +1609,14 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Podcast Rec: Coaching for Leaders with Dave Stachowiak</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>https://coachingforleaders.com/</t>
-        </is>
-      </c>
+          <t>93.75% Rated Excellent at ASBA 2025</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Podcast Recommendation</t>
+          <t>Stats and Proof</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1691,17 +1628,14 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>The Personal Histories Exercise</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/personal-histories-exercise</t>
-        </is>
-      </c>
+          <t>Signs Your Executive Team is Dysfunctional</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Blog Post</t>
+          <t>Blog</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1713,17 +1647,14 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Book Rec: The Ideal Team Player by Patrick Lencioni</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>https://www.tablegroup.com/the-ideal-team-player/</t>
-        </is>
-      </c>
+          <t>Book Rec: Extreme Ownership by Jocko Willink</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Book Recommendation</t>
+          <t>Book Rec</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1735,17 +1666,14 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Podcast Rec: Global Leadership Summit Podcast</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>https://globalleadership.org/podcast/</t>
-        </is>
-      </c>
+          <t>The Meeting That Went Perfectly Is the One to Worry About</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Podcast Recommendation</t>
+          <t>Pain Point</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1757,17 +1685,14 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>The Thematic Goal: A Lencioni Guide</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/thematic-goal-lencioni-guide</t>
-        </is>
-      </c>
+          <t>Podcast Rec: The Learning Leader Show with Ryan Hawk</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Blog Post</t>
+          <t>Podcast Rec</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1779,17 +1704,14 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Book Rec: Multipliers by Liz Wiseman</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>https://thewisemangroup.com/books/multipliers/</t>
-        </is>
-      </c>
+          <t>Testimonial: Edward Amey, USA</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Book Recommendation</t>
+          <t>Testimonial</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1801,17 +1723,14 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Podcast Rec: Lead to Win with Michael Hyatt</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>https://fullfocus.co/podcast/</t>
-        </is>
-      </c>
+          <t>Service: Executive Coaching for Leaders</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Podcast Recommendation</t>
+          <t>Service</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1823,17 +1742,14 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Leadership Lessons from JFK</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>https://www.consultclarity.org/post/leadership-lessons-jfk</t>
-        </is>
-      </c>
+          <t>Working Genius: 6 Types That Energise or Drain You</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Blog Post</t>
+          <t>Framework</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1845,17 +1761,14 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Book Rec: Grit by Angela Duckworth</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>https://angeladuckworth.com/grit-book/</t>
-        </is>
-      </c>
+          <t>The Five Dysfunctions of a Team (Summary)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Book Recommendation</t>
+          <t>Blog</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1867,20 +1780,2107 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>Book Rec: Crucial Conversations by Patterson et al</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Your Best Teacher Just Resigned</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Dare to Lead with Brene Brown</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr"/>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Testimonial: Tim Chalmers, Australia</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr"/>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Service: Board Offsite for Nonprofits</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>The Pre-Brief Zoom Call That Creates 80% of the Value</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr"/>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Vulnerability-Based Trust</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr"/>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Book Rec: Atomic Habits by James Clear</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>We Did an Offsite and Nothing Changed</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Podcast Rec: The John Maxwell Leadership Podcast</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Testimonial: Emily Hynes, Australia</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Service: Strategic Planning Facilitation</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr"/>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>10000+ Copies of Step Up or Step Out Sold Globally</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr"/>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Tips for Your First Year as Principal</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr"/>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Book Rec: Hidden Potential by Adam Grant</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr"/>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Talented Individually Dysfunctional Together</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr"/>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Coaching for Leaders with Dave Stachowiak</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr"/>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Testimonial: Ian Cumming, Australia</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Service: School Leadership PD Day</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Step Up or Step Out: The Framework</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>The Personal Histories Exercise</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Book Rec: The Ideal Team Player by Patrick Lencioni</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Nobody Has Energy for Execution</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Global Leadership Summit Podcast</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Testimonial: Nita Davis, USA</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Service: Working Genius for Hiring</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>What a Leadership Team Offsite Actually Looks Like</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>The Thematic Goal: A Lencioni Guide</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr"/>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Book Rec: Multipliers by Liz Wiseman</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr"/>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>The Quietest Person Is the Most Important</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr"/>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Lead to Win with Michael Hyatt</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr"/>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Testimonial: Mike Pieper, USA</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr"/>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Service: Leadership Team Offsite for Hospitals</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr"/>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>230+ Episodes of The Leadership Conversations Podcast</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Leadership Lessons from JFK</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr"/>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Book Rec: Grit by Angela Duckworth</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Conference Evals Are Fine But They Are Not Coming Back</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
           <t>Podcast Rec: EntreLeadership Podcast by Ramsey Solutions</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>https://www.ramseysolutions.com/shows/the-entreleadership-podcast</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Podcast Recommendation</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Testimonial: Jessica Morrow, USA</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr"/>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Service: MC and Hosting for Events</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr"/>
+      <c r="C87" t="inlineStr"/>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>The Thematic Goal: How to Align Your Team</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr"/>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>How to Run an Effective Leadership Team Offsite</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr"/>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Book Rec: The Five Dysfunctions of a Team by Lencioni</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr"/>
+      <c r="C90" t="inlineStr"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>My Board Wants Strategy But My Team Is Burnt Out</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr"/>
+      <c r="C91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Better Leaders Better Schools with Danny Bauer</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr"/>
+      <c r="C92" t="inlineStr"/>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Testimonial: Jonathan Price, New Zealand</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr"/>
+      <c r="C93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Service: DISC Workshop for Teams</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr"/>
+      <c r="C94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>How I Design a Keynote</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr"/>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Why Great Leaders Ask Better Questions</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr"/>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Book Rec: Good to Great by Jim Collins</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr"/>
+      <c r="C97" t="inlineStr"/>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Your Brilliant Jerk Costs More Than Your Best Hire</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr"/>
+      <c r="C98" t="inlineStr"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Podcast Rec: No Bullshit Leadership with Martin G. Moore</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr"/>
+      <c r="C99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Testimonial: Graeme Budler, New Zealand</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr"/>
+      <c r="C100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Service: Working Genius for Nonprofits</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr"/>
+      <c r="C101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>6000+ Leaders in The 7 Questions Movement</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr"/>
+      <c r="C102" t="inlineStr"/>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Building Trust in Remote Leadership Teams</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr"/>
+      <c r="C103" t="inlineStr"/>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Book Rec: The Coaching Habit by Michael Bungay Stanier</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr"/>
+      <c r="C104" t="inlineStr"/>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Podcast Rec: The Ed Mylett Show</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr"/>
+      <c r="C105" t="inlineStr"/>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Testimonial: Trent Raddatz, Australia</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr"/>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Service: Leadership Offsite for Schools</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr"/>
+      <c r="C107" t="inlineStr"/>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Trust Starts with Vulnerability</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr"/>
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>The Hidden Cost of Avoiding Difficult Conversations</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr"/>
+      <c r="C109" t="inlineStr"/>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Book Rec: Dare to Lead by Brene Brown</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr"/>
+      <c r="C110" t="inlineStr"/>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Podcast Rec: How Leaders Lead with David Novak</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr"/>
+      <c r="C111" t="inlineStr"/>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Testimonial: Lyndall Waters, Australia</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr"/>
+      <c r="C112" t="inlineStr"/>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Service: StrengthsFinder Session</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr"/>
+      <c r="C113" t="inlineStr"/>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>The Debrief 48 Hours After a Session</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr"/>
+      <c r="C114" t="inlineStr"/>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Why Your Strategic Plan Is Collecting Dust</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr"/>
+      <c r="C115" t="inlineStr"/>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Book Rec: Start with Why by Simon Sinek</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr"/>
+      <c r="C116" t="inlineStr"/>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Podcast Rec: School Leadership Reimagined</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr"/>
+      <c r="C117" t="inlineStr"/>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Testimonial: Nathan Gilmour, Australia</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr"/>
+      <c r="C118" t="inlineStr"/>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Service: Executive Coaching for Principals</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr"/>
+      <c r="C119" t="inlineStr"/>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>1.3 Million People Have Taken Working Genius</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr"/>
+      <c r="C120" t="inlineStr"/>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>How to Create Psychological Safety in Schools</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr"/>
+      <c r="C121" t="inlineStr"/>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Book Rec: The Culture Code by Daniel Coyle</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr"/>
+      <c r="C122" t="inlineStr"/>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Andy Stanley Leadership Podcast</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr"/>
+      <c r="C123" t="inlineStr"/>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Testimonial: Christopher Martin, New Zealand</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr"/>
+      <c r="C124" t="inlineStr"/>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>How to Run a Meeting Your Team Doesn't Dread</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr"/>
+      <c r="C125" t="inlineStr"/>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>The Problem with Performance Reviews</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr"/>
+      <c r="C126" t="inlineStr"/>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Book Rec: Turn the Ship Around by L. David Marquet</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr"/>
+      <c r="C127" t="inlineStr"/>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Podcast Rec: At the Table with Patrick Lencioni</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr"/>
+      <c r="C128" t="inlineStr"/>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Testimonial: Colette Budler, New Zealand</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr"/>
+      <c r="C129" t="inlineStr"/>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>How I Use Working Genius and DISC Together</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr"/>
+      <c r="C130" t="inlineStr"/>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>What New CEOs Get Wrong in Their First 90 Days</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr"/>
+      <c r="C131" t="inlineStr"/>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Book Rec: Team of Teams by Stanley McChrystal</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr"/>
+      <c r="C132" t="inlineStr"/>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Podcast Rec: The Maxwell Leadership Podcast</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr"/>
+      <c r="C133" t="inlineStr"/>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Testimonial: Paul Thompson, Australia</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr"/>
+      <c r="C134" t="inlineStr"/>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>The Ideal Team Player: Humble Hungry Smart</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr"/>
+      <c r="C135" t="inlineStr"/>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Why Culture Eats Strategy for Breakfast</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr"/>
+      <c r="C136" t="inlineStr"/>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Book Rec: No Bullshit Leadership by Martin G. Moore</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr"/>
+      <c r="C137" t="inlineStr"/>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Testimonial: Jonathan Burnett, Australia</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr"/>
+      <c r="C138" t="inlineStr"/>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>What the First Coaching Session Looks Like</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr"/>
+      <c r="C139" t="inlineStr"/>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>How to Build a Leadership Pipeline in Schools</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr"/>
+      <c r="C140" t="inlineStr"/>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Book Rec: Blindspotting by Kirstin Ferguson</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr"/>
+      <c r="C141" t="inlineStr"/>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Testimonial: Lucie Wiradjaja, Australia</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr"/>
+      <c r="C142" t="inlineStr"/>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>The Personal Histories Exercise Explained</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr"/>
+      <c r="C143" t="inlineStr"/>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>The 7 Questions Every Leader Should Ask Their Team</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr"/>
+      <c r="C144" t="inlineStr"/>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Book Rec: The Advantage by Patrick Lencioni</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr"/>
+      <c r="C145" t="inlineStr"/>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Testimonial: Julie Edds, Australia</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr"/>
+      <c r="C146" t="inlineStr"/>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>When Your Best People Start Leaving</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr"/>
+      <c r="C147" t="inlineStr"/>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Book Rec: Death by Meeting by Patrick Lencioni</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr"/>
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Testimonial: Amber Wilson, Australia</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr"/>
+      <c r="C149" t="inlineStr"/>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>How to Facilitate a Meeting That Produces Decisions</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr"/>
+      <c r="C150" t="inlineStr"/>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Book Rec: Drive by Daniel Pink</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr"/>
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Testimonial: Claire Whereat, Australia</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr"/>
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>The Difference Between a Group and a Team</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr"/>
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Book Rec: Thinking Fast and Slow by Daniel Kahneman</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr"/>
+      <c r="C154" t="inlineStr"/>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Testimonial: James Norman, Australia</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr"/>
+      <c r="C155" t="inlineStr"/>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Why Most Team Building Activities Don't Work</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr"/>
+      <c r="C156" t="inlineStr"/>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Book Rec: Storyworthy by Matthew Dicks</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr"/>
+      <c r="C157" t="inlineStr"/>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Testimonial: Dirk Lategan, Australia</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr"/>
+      <c r="C158" t="inlineStr"/>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after caring-hurts-leadership run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1232,8 +1232,11 @@
           <t>Caring Hurts: The Hidden Cost of Leadership</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/caring-hurts-leadership</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -1241,7 +1244,32 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>why-caring-hurts, signs-1-to-5, signs-6-to-10, caring-that-builds</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>8, 7, 7, 8</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>4 carousels from blog post. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>
@@ -1251,8 +1279,6 @@
           <t>Book Rec: Leaders Eat Last by Simon Sinek</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -1270,8 +1296,6 @@
           <t>My Team Nods But Nothing Changes</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
           <t>Pain Point</t>
@@ -1289,8 +1313,6 @@
           <t>Podcast Rec: Craig Groeschel Leadership Podcast</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -1308,8 +1330,6 @@
           <t>Testimonial: Kathy Dickson, CEO ASBA</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -1327,8 +1347,6 @@
           <t>Service: Leadership Team Offsite for Corporates</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
           <t>Service</t>
@@ -1346,8 +1364,6 @@
           <t>The 5 Dysfunctions of a Team Explained</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
           <t>Framework</t>
@@ -1365,8 +1381,6 @@
           <t>Imposter Syndrome as a Leader</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -1384,8 +1398,6 @@
           <t>Book Rec: Unreasonable Hospitality by Will Guidara</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -1403,8 +1415,6 @@
           <t>We Keep Losing Good Teachers</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
           <t>Pain Point</t>
@@ -1422,8 +1432,6 @@
           <t>Podcast Rec: HBR IdeaCast</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -1441,8 +1449,6 @@
           <t>Testimonial: Michael Quach, Redlands College</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -1460,8 +1466,6 @@
           <t>Service: Working Genius Workshop for Schools</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
           <t>Service</t>
@@ -1479,8 +1483,6 @@
           <t>What Actually Happens in a Working Genius Session</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
           <t>Behind the Scenes</t>
@@ -1498,8 +1500,6 @@
           <t>Leading Through Uncertainty</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -1517,8 +1517,6 @@
           <t>Book Rec: Radical Candor by Kim Scott</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
       <c r="D34" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -1536,8 +1534,6 @@
           <t>Every Year We Set Priorities and Do the Same Things</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>Pain Point</t>
@@ -1555,8 +1551,6 @@
           <t>Podcast Rec: WorkLife with Adam Grant</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -1574,8 +1568,6 @@
           <t>Testimonial: Brett Bleakley, Livingstone Christian School</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -1593,8 +1585,6 @@
           <t>Service: Keynote Speaking for Conferences</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
           <t>Service</t>
@@ -1612,8 +1602,6 @@
           <t>93.75% Rated Excellent at ASBA 2025</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
       <c r="D39" t="inlineStr">
         <is>
           <t>Stats and Proof</t>
@@ -1631,8 +1619,6 @@
           <t>Signs Your Executive Team is Dysfunctional</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -1650,8 +1636,6 @@
           <t>Book Rec: Extreme Ownership by Jocko Willink</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -1669,8 +1653,6 @@
           <t>The Meeting That Went Perfectly Is the One to Worry About</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>Pain Point</t>
@@ -1688,8 +1670,6 @@
           <t>Podcast Rec: The Learning Leader Show with Ryan Hawk</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
       <c r="D43" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -1707,8 +1687,6 @@
           <t>Testimonial: Edward Amey, USA</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -1726,8 +1704,6 @@
           <t>Service: Executive Coaching for Leaders</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
       <c r="D45" t="inlineStr">
         <is>
           <t>Service</t>
@@ -1745,8 +1721,6 @@
           <t>Working Genius: 6 Types That Energise or Drain You</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
       <c r="D46" t="inlineStr">
         <is>
           <t>Framework</t>
@@ -1764,8 +1738,6 @@
           <t>The Five Dysfunctions of a Team (Summary)</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
       <c r="D47" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -1783,8 +1755,6 @@
           <t>Book Rec: Crucial Conversations by Patterson et al</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -1802,8 +1772,6 @@
           <t>Your Best Teacher Just Resigned</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
       <c r="D49" t="inlineStr">
         <is>
           <t>Pain Point</t>
@@ -1821,8 +1789,6 @@
           <t>Podcast Rec: Dare to Lead with Brene Brown</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
       <c r="D50" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -1840,8 +1806,6 @@
           <t>Testimonial: Tim Chalmers, Australia</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -1859,8 +1823,6 @@
           <t>Service: Board Offsite for Nonprofits</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
       <c r="D52" t="inlineStr">
         <is>
           <t>Service</t>
@@ -1878,8 +1840,6 @@
           <t>The Pre-Brief Zoom Call That Creates 80% of the Value</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
       <c r="D53" t="inlineStr">
         <is>
           <t>Behind the Scenes</t>
@@ -1897,8 +1857,6 @@
           <t>Vulnerability-Based Trust</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -1916,8 +1874,6 @@
           <t>Book Rec: Atomic Habits by James Clear</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -1935,8 +1891,6 @@
           <t>We Did an Offsite and Nothing Changed</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
       <c r="D56" t="inlineStr">
         <is>
           <t>Pain Point</t>
@@ -1954,8 +1908,6 @@
           <t>Podcast Rec: The John Maxwell Leadership Podcast</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -1973,8 +1925,6 @@
           <t>Testimonial: Emily Hynes, Australia</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr"/>
       <c r="D58" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -1992,8 +1942,6 @@
           <t>Service: Strategic Planning Facilitation</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
       <c r="D59" t="inlineStr">
         <is>
           <t>Service</t>
@@ -2011,8 +1959,6 @@
           <t>10000+ Copies of Step Up or Step Out Sold Globally</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
       <c r="D60" t="inlineStr">
         <is>
           <t>Stats and Proof</t>
@@ -2030,8 +1976,6 @@
           <t>Tips for Your First Year as Principal</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
       <c r="D61" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -2049,8 +1993,6 @@
           <t>Book Rec: Hidden Potential by Adam Grant</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
       <c r="D62" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -2068,8 +2010,6 @@
           <t>Talented Individually Dysfunctional Together</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr"/>
       <c r="D63" t="inlineStr">
         <is>
           <t>Pain Point</t>
@@ -2087,8 +2027,6 @@
           <t>Podcast Rec: Coaching for Leaders with Dave Stachowiak</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr"/>
       <c r="D64" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -2106,8 +2044,6 @@
           <t>Testimonial: Ian Cumming, Australia</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -2125,8 +2061,6 @@
           <t>Service: School Leadership PD Day</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr">
         <is>
           <t>Service</t>
@@ -2144,8 +2078,6 @@
           <t>Step Up or Step Out: The Framework</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr"/>
       <c r="D67" t="inlineStr">
         <is>
           <t>Framework</t>
@@ -2163,8 +2095,6 @@
           <t>The Personal Histories Exercise</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -2182,8 +2112,6 @@
           <t>Book Rec: The Ideal Team Player by Patrick Lencioni</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr"/>
       <c r="D69" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -2201,8 +2129,6 @@
           <t>Nobody Has Energy for Execution</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
       <c r="D70" t="inlineStr">
         <is>
           <t>Pain Point</t>
@@ -2220,8 +2146,6 @@
           <t>Podcast Rec: Global Leadership Summit Podcast</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
       <c r="D71" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -2239,8 +2163,6 @@
           <t>Testimonial: Nita Davis, USA</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -2258,8 +2180,6 @@
           <t>Service: Working Genius for Hiring</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr">
         <is>
           <t>Service</t>
@@ -2277,8 +2197,6 @@
           <t>What a Leadership Team Offsite Actually Looks Like</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr"/>
       <c r="D74" t="inlineStr">
         <is>
           <t>Behind the Scenes</t>
@@ -2296,8 +2214,6 @@
           <t>The Thematic Goal: A Lencioni Guide</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -2315,8 +2231,6 @@
           <t>Book Rec: Multipliers by Liz Wiseman</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr"/>
       <c r="D76" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -2334,8 +2248,6 @@
           <t>The Quietest Person Is the Most Important</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
-      <c r="C77" t="inlineStr"/>
       <c r="D77" t="inlineStr">
         <is>
           <t>Pain Point</t>
@@ -2353,8 +2265,6 @@
           <t>Podcast Rec: Lead to Win with Michael Hyatt</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -2372,8 +2282,6 @@
           <t>Testimonial: Mike Pieper, USA</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr"/>
       <c r="D79" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -2391,8 +2299,6 @@
           <t>Service: Leadership Team Offsite for Hospitals</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
           <t>Service</t>
@@ -2410,8 +2316,6 @@
           <t>230+ Episodes of The Leadership Conversations Podcast</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr"/>
       <c r="D81" t="inlineStr">
         <is>
           <t>Stats and Proof</t>
@@ -2429,8 +2333,6 @@
           <t>Leadership Lessons from JFK</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr"/>
       <c r="D82" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -2448,8 +2350,6 @@
           <t>Book Rec: Grit by Angela Duckworth</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -2467,8 +2367,6 @@
           <t>Conference Evals Are Fine But They Are Not Coming Back</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr"/>
       <c r="D84" t="inlineStr">
         <is>
           <t>Pain Point</t>
@@ -2486,8 +2384,6 @@
           <t>Podcast Rec: EntreLeadership Podcast by Ramsey Solutions</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
-      <c r="C85" t="inlineStr"/>
       <c r="D85" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -2505,8 +2401,6 @@
           <t>Testimonial: Jessica Morrow, USA</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr"/>
       <c r="D86" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -2524,8 +2418,6 @@
           <t>Service: MC and Hosting for Events</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
-      <c r="C87" t="inlineStr"/>
       <c r="D87" t="inlineStr">
         <is>
           <t>Service</t>
@@ -2543,8 +2435,6 @@
           <t>The Thematic Goal: How to Align Your Team</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr"/>
       <c r="D88" t="inlineStr">
         <is>
           <t>Framework</t>
@@ -2562,8 +2452,6 @@
           <t>How to Run an Effective Leadership Team Offsite</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
-      <c r="C89" t="inlineStr"/>
       <c r="D89" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -2581,8 +2469,6 @@
           <t>Book Rec: The Five Dysfunctions of a Team by Lencioni</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
-      <c r="C90" t="inlineStr"/>
       <c r="D90" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -2600,8 +2486,6 @@
           <t>My Board Wants Strategy But My Team Is Burnt Out</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
-      <c r="C91" t="inlineStr"/>
       <c r="D91" t="inlineStr">
         <is>
           <t>Pain Point</t>
@@ -2619,8 +2503,6 @@
           <t>Podcast Rec: Better Leaders Better Schools with Danny Bauer</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
-      <c r="C92" t="inlineStr"/>
       <c r="D92" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -2638,8 +2520,6 @@
           <t>Testimonial: Jonathan Price, New Zealand</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr"/>
       <c r="D93" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -2657,8 +2537,6 @@
           <t>Service: DISC Workshop for Teams</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
-      <c r="C94" t="inlineStr"/>
       <c r="D94" t="inlineStr">
         <is>
           <t>Service</t>
@@ -2676,8 +2554,6 @@
           <t>How I Design a Keynote</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr"/>
       <c r="D95" t="inlineStr">
         <is>
           <t>Behind the Scenes</t>
@@ -2695,8 +2571,6 @@
           <t>Why Great Leaders Ask Better Questions</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr"/>
       <c r="D96" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -2714,8 +2588,6 @@
           <t>Book Rec: Good to Great by Jim Collins</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
       <c r="D97" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -2733,8 +2605,6 @@
           <t>Your Brilliant Jerk Costs More Than Your Best Hire</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr"/>
-      <c r="C98" t="inlineStr"/>
       <c r="D98" t="inlineStr">
         <is>
           <t>Pain Point</t>
@@ -2752,8 +2622,6 @@
           <t>Podcast Rec: No Bullshit Leadership with Martin G. Moore</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr"/>
-      <c r="C99" t="inlineStr"/>
       <c r="D99" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -2771,8 +2639,6 @@
           <t>Testimonial: Graeme Budler, New Zealand</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr"/>
-      <c r="C100" t="inlineStr"/>
       <c r="D100" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -2790,8 +2656,6 @@
           <t>Service: Working Genius for Nonprofits</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr"/>
-      <c r="C101" t="inlineStr"/>
       <c r="D101" t="inlineStr">
         <is>
           <t>Service</t>
@@ -2809,8 +2673,6 @@
           <t>6000+ Leaders in The 7 Questions Movement</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr"/>
-      <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
           <t>Stats and Proof</t>
@@ -2828,8 +2690,6 @@
           <t>Building Trust in Remote Leadership Teams</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr"/>
-      <c r="C103" t="inlineStr"/>
       <c r="D103" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -2847,8 +2707,6 @@
           <t>Book Rec: The Coaching Habit by Michael Bungay Stanier</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr"/>
-      <c r="C104" t="inlineStr"/>
       <c r="D104" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -2866,8 +2724,6 @@
           <t>Podcast Rec: The Ed Mylett Show</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr"/>
-      <c r="C105" t="inlineStr"/>
       <c r="D105" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -2885,8 +2741,6 @@
           <t>Testimonial: Trent Raddatz, Australia</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr"/>
-      <c r="C106" t="inlineStr"/>
       <c r="D106" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -2904,8 +2758,6 @@
           <t>Service: Leadership Offsite for Schools</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr"/>
-      <c r="C107" t="inlineStr"/>
       <c r="D107" t="inlineStr">
         <is>
           <t>Service</t>
@@ -2923,8 +2775,6 @@
           <t>Trust Starts with Vulnerability</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr"/>
-      <c r="C108" t="inlineStr"/>
       <c r="D108" t="inlineStr">
         <is>
           <t>Framework</t>
@@ -2942,8 +2792,6 @@
           <t>The Hidden Cost of Avoiding Difficult Conversations</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr"/>
-      <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -2961,8 +2809,6 @@
           <t>Book Rec: Dare to Lead by Brene Brown</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr"/>
-      <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -2980,8 +2826,6 @@
           <t>Podcast Rec: How Leaders Lead with David Novak</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr"/>
-      <c r="C111" t="inlineStr"/>
       <c r="D111" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -2999,8 +2843,6 @@
           <t>Testimonial: Lyndall Waters, Australia</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr"/>
-      <c r="C112" t="inlineStr"/>
       <c r="D112" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -3018,8 +2860,6 @@
           <t>Service: StrengthsFinder Session</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr"/>
-      <c r="C113" t="inlineStr"/>
       <c r="D113" t="inlineStr">
         <is>
           <t>Service</t>
@@ -3037,8 +2877,6 @@
           <t>The Debrief 48 Hours After a Session</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr"/>
-      <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr">
         <is>
           <t>Behind the Scenes</t>
@@ -3056,8 +2894,6 @@
           <t>Why Your Strategic Plan Is Collecting Dust</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr"/>
-      <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -3075,8 +2911,6 @@
           <t>Book Rec: Start with Why by Simon Sinek</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr"/>
-      <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -3094,8 +2928,6 @@
           <t>Podcast Rec: School Leadership Reimagined</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr"/>
-      <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -3113,8 +2945,6 @@
           <t>Testimonial: Nathan Gilmour, Australia</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr"/>
-      <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -3132,8 +2962,6 @@
           <t>Service: Executive Coaching for Principals</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr"/>
-      <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr">
         <is>
           <t>Service</t>
@@ -3151,8 +2979,6 @@
           <t>1.3 Million People Have Taken Working Genius</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr"/>
-      <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr">
         <is>
           <t>Stats and Proof</t>
@@ -3170,8 +2996,6 @@
           <t>How to Create Psychological Safety in Schools</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr"/>
-      <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -3189,8 +3013,6 @@
           <t>Book Rec: The Culture Code by Daniel Coyle</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr"/>
-      <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -3208,8 +3030,6 @@
           <t>Podcast Rec: Andy Stanley Leadership Podcast</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
-      <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -3227,8 +3047,6 @@
           <t>Testimonial: Christopher Martin, New Zealand</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr"/>
-      <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -3246,8 +3064,6 @@
           <t>How to Run a Meeting Your Team Doesn't Dread</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr"/>
-      <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr">
         <is>
           <t>Framework</t>
@@ -3265,8 +3081,6 @@
           <t>The Problem with Performance Reviews</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr"/>
-      <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -3284,8 +3098,6 @@
           <t>Book Rec: Turn the Ship Around by L. David Marquet</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr"/>
-      <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -3303,8 +3115,6 @@
           <t>Podcast Rec: At the Table with Patrick Lencioni</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr"/>
-      <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -3322,8 +3132,6 @@
           <t>Testimonial: Colette Budler, New Zealand</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr"/>
-      <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -3341,8 +3149,6 @@
           <t>How I Use Working Genius and DISC Together</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr"/>
-      <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr">
         <is>
           <t>Behind the Scenes</t>
@@ -3360,8 +3166,6 @@
           <t>What New CEOs Get Wrong in Their First 90 Days</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr"/>
-      <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -3379,8 +3183,6 @@
           <t>Book Rec: Team of Teams by Stanley McChrystal</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr"/>
-      <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -3398,8 +3200,6 @@
           <t>Podcast Rec: The Maxwell Leadership Podcast</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr"/>
-      <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr">
         <is>
           <t>Podcast Rec</t>
@@ -3417,8 +3217,6 @@
           <t>Testimonial: Paul Thompson, Australia</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr"/>
-      <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -3436,8 +3234,6 @@
           <t>The Ideal Team Player: Humble Hungry Smart</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr"/>
-      <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr">
         <is>
           <t>Framework</t>
@@ -3455,8 +3251,6 @@
           <t>Why Culture Eats Strategy for Breakfast</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr"/>
-      <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -3474,8 +3268,6 @@
           <t>Book Rec: No Bullshit Leadership by Martin G. Moore</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr"/>
-      <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -3493,8 +3285,6 @@
           <t>Testimonial: Jonathan Burnett, Australia</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr"/>
-      <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -3512,8 +3302,6 @@
           <t>What the First Coaching Session Looks Like</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr"/>
-      <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr">
         <is>
           <t>Behind the Scenes</t>
@@ -3531,8 +3319,6 @@
           <t>How to Build a Leadership Pipeline in Schools</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr"/>
-      <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -3550,8 +3336,6 @@
           <t>Book Rec: Blindspotting by Kirstin Ferguson</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr"/>
-      <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -3569,8 +3353,6 @@
           <t>Testimonial: Lucie Wiradjaja, Australia</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr"/>
-      <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -3588,8 +3370,6 @@
           <t>The Personal Histories Exercise Explained</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr"/>
-      <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr">
         <is>
           <t>Framework</t>
@@ -3607,8 +3387,6 @@
           <t>The 7 Questions Every Leader Should Ask Their Team</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr"/>
-      <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -3626,8 +3404,6 @@
           <t>Book Rec: The Advantage by Patrick Lencioni</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr"/>
-      <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -3645,8 +3421,6 @@
           <t>Testimonial: Julie Edds, Australia</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr"/>
-      <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -3664,8 +3438,6 @@
           <t>When Your Best People Start Leaving</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr"/>
-      <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -3683,8 +3455,6 @@
           <t>Book Rec: Death by Meeting by Patrick Lencioni</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr"/>
-      <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -3702,8 +3472,6 @@
           <t>Testimonial: Amber Wilson, Australia</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr"/>
-      <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -3721,8 +3489,6 @@
           <t>How to Facilitate a Meeting That Produces Decisions</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr"/>
-      <c r="C150" t="inlineStr"/>
       <c r="D150" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -3740,8 +3506,6 @@
           <t>Book Rec: Drive by Daniel Pink</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr"/>
-      <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -3759,8 +3523,6 @@
           <t>Testimonial: Claire Whereat, Australia</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr"/>
-      <c r="C152" t="inlineStr"/>
       <c r="D152" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -3778,8 +3540,6 @@
           <t>The Difference Between a Group and a Team</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr"/>
-      <c r="C153" t="inlineStr"/>
       <c r="D153" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -3797,8 +3557,6 @@
           <t>Book Rec: Thinking Fast and Slow by Daniel Kahneman</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr"/>
-      <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -3816,8 +3574,6 @@
           <t>Testimonial: James Norman, Australia</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr"/>
-      <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr">
         <is>
           <t>Testimonial</t>
@@ -3835,8 +3591,6 @@
           <t>Why Most Team Building Activities Don't Work</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr"/>
-      <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -3854,8 +3608,6 @@
           <t>Book Rec: Storyworthy by Matthew Dicks</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr"/>
-      <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr">
         <is>
           <t>Book Rec</t>
@@ -3873,8 +3625,6 @@
           <t>Testimonial: Dirk Lategan, Australia</t>
         </is>
       </c>
-      <c r="B158" t="inlineStr"/>
-      <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr">
         <is>
           <t>Testimonial</t>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after Leaders Eat Last carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1286,7 +1286,32 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>why-read-leaders-eat-last, circle-of-safety, four-chemicals-of-leadership, key-lessons-leaders-eat-last</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>8, 8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Book rec post. 4 carousels covering overview, Circle of Safety, 4 chemicals, key lessons.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after carousel run - Craig Groeschel Podcast
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1370,7 +1370,32 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Why Listen to Craig Groeschel, 5 Key Themes, 3 Reasons to Subscribe</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>8, 7, 6</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Pinterest skipped (no boards)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after ASBA testimonial carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1412,7 +1412,32 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>asba-working-genius-in-action, asba-93-percent-rated-excellent, asba-what-school-leaders-took-away</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>7, 7, 7</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>3 carousels from ASBA testimonial. TikTok/YouTube hit daily Buffer limits. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after carousel run - offsite corporates
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1454,7 +1454,32 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>offsite-why-your-team-needs-one, offsite-what-to-expect, offsite-common-mistakes, offsite-book-your-offsite</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>8, 8, 8, 7</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>4 carousels from service page. Pinterest skipped (no boards). YouTube Apr 11-14. TikTok May 8-11.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after Topic 1
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1496,7 +1496,32 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>5-dysfunctions-overview, 5-dysfunctions-trust-conflict, 5-dysfunctions-commitment-results, 5-dysfunctions-action-plan</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>9, 8, 9, 8</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>4 carousels from framework topic. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after Topic 2
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1538,7 +1538,32 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>imposter-syndrome-signs, imposter-syndrome-cost, imposter-syndrome-overcome</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>3 carousels from blog topic. Pinterest skipped.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx after Topic 3
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1580,7 +1580,32 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>unreasonable-hospitality-why-read, unreasonable-hospitality-lessons, unreasonable-hospitality-apply</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>7, 7, 7</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>3 carousels from book rec. Pinterest skipped.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx - session complete (4 topics)
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1622,7 +1622,32 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>losing-teachers-warning-signs, losing-teachers-real-reasons, losing-teachers-what-to-do</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>8, 8, 7</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>3 carousels from pain point topic. Pinterest skipped.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx - Topic 2 Redlands College
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1706,7 +1706,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>redlands-wg-overview, redlands-wg-discoveries, redlands-wg-book-session</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx - Topic 3 Schools WG
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1733,7 +1733,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>schools-wg-why, schools-wg-how, schools-wg-transform</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx - Topic 4 WG Session
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1760,7 +1760,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>wg-session-inside, wg-session-moments, wg-session-book</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - Topic 1
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1787,7 +1787,32 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>understanding-uncertainty, decision-making-uncertainty, communication-trust-uncertainty, resilience-adaptive-strategy</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>8, 8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>4 carousels from blog post. All 9 platforms scheduled. YouTube Apr 15-18. TikTok Mar 30-31.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar after Topic 1
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1871,7 +1871,32 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>why-priorities-fail, signs-plan-will-fail, break-the-cycle</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>8, 7, 8</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>LI, FB, IG, Threads, X, GBP, TikTok, YT, Bluesky (carousel 3: 5 platforms failed duplicate detection)</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Pain point topic. 3 carousels. Carousel 3 blocked by Buffer duplicate detection on LI/FB/Threads/X/Bluesky.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar: Topic 2 WorkLife with Adam Grant
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1913,7 +1913,32 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>worklife-podcast-rec, worklife-why-listen</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2 carousels. All 9 platforms scheduled successfully.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar: Topics 3-4 (keynote speaking + exec dysfunction)
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -1955,7 +1955,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>No testimonial content found online. Needs manual input of testimonial text.</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1977,32 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>keynote-speaking-service, why-book-jonno</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2 carousels. All 9 platforms scheduled successfully.</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2036,32 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>exec-team-dysfunction, fix-dysfunctional-team</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>9, 7</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok, YouTube</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2 carousels. All 9 platforms scheduled successfully. Based on Lencioni's Five Dysfunctions.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - Topic 1 ASBA proof
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2019,7 +2019,32 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>asba-93-percent-proof, asba-what-makes-pd-great</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2 carousels. YouTube and Google Business disconnected. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - Topic 2 Extreme Ownership
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2103,7 +2103,32 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>extreme-ownership-why-read, extreme-ownership-principles, extreme-ownership-apply</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>8, 8, 7</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>3 carousels. YouTube and Google Business disconnected. Pinterest skipped.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar - Topic 3 meeting perfect
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2145,7 +2145,32 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>perfect-meeting-danger, perfect-meeting-fix</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Pain point topic. YouTube/Google Business disconnected. TikTok scheduled May 25-26.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar - Topic 4 Learning Leader
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2187,7 +2187,32 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>learning-leader-rec, learning-leader-lessons</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Bluesky, TikTok</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Podcast rec for Ryan Hawk. YouTube/Google Business disconnected. TikTok scheduled May 27-28.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx - Topic 1: Edward Amey testimonial
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -59,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2229,7 +2232,30 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>offsite-insights-edward-amey, leadership-disability-edward-amey</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>No specific testimonial quote found. Built carousels from verified podcast content (EP225) and public bio.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx - Topic 2: Executive Coaching
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2272,7 +2272,30 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>why-leaders-need-a-coach, what-coaching-looks-like, cost-of-no-coach</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Service promo carousel. No people tagged.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx - Topic 1 Working Genius
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2312,7 +2312,32 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>wg-6-types, wg-genius-or-frustration, wg-transforms-teams</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>All 9 platforms scheduled. YouTube on Apr 15-17 due to daily limits.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx - Topic 2 Five Dysfunctions
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2354,7 +2354,32 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>5d-overview, 5d-overcome, 5d-warning-signs</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>All 9 platforms scheduled. YouTube on Apr 18-20.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - Crucial Conversations
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2396,7 +2396,32 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>crucial-conversations-why-read, crucial-conversations-7-skills, crucial-conversations-apply</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>8, 9, 8</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Book rec. 3 carousels. All 9 platforms. YouTube Apr 28-30. TikTok Jun 9-11. Pinterest skipped (no boards).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - Board Offsite Nonprofits
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2522,7 +2522,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>No testimonial content found online. Needs manual input of testimonial text.</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2544,32 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>board-offsite-why, board-offsite-5-signs</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>8, 7</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Service topic. No blog URL. 2 carousels. Tim Chalmers row skipped (no content found).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - Topic 1 pre-brief
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2586,7 +2586,32 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>pre-brief-call, 5-questions-before-offsite</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Behind the scenes content. No people to tag.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - Topic 2 VBT
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2621,6 +2621,11 @@
           <t>Vulnerability-Based Trust</t>
         </is>
       </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://www.consultclarity.org/post/vulnerability-based-trust</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr">
         <is>
           <t>Blog</t>
@@ -2628,7 +2633,32 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>what-is-vulnerability-based-trust, 7-ways-vulnerability-trust, leader-must-go-first</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>8, 9, 8</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Blog post carousel. 3 carousels from Lencioni VBT concept.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar: Topic 2 Maxwell Podcast done
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2759,7 +2759,32 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>maxwell-podcast-why-listen, maxwell-podcast-key-themes</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Podcast rec. TikTok Jun 21, YouTube Jun 12.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar: Topic 3 Strategic Planning done
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2823,7 +2823,32 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>strategic-plan-why-facilitator, strategic-plan-5-signs-dust</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Service topic. TikTok Jun 22-23, YouTube Jun 13-14.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Final update: all 4 topics complete
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2865,7 +2865,32 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>step-up-10k-milestone, step-up-3-stages</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>8, 8</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Book milestone. TikTok Jun 24-25, YouTube Jun 15-16.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - Topic 1 done
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2907,7 +2907,32 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>build-relationships-first, avoid-common-mistakes, lead-instruction-with-confidence</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>No blog URL. Content researched from web. School topic, used WG Facilitator footer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 200 new content calendar rows (rows 159-358)
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J158"/>
+  <dimension ref="A1:J358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2907,32 +2907,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Carousel Created</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>2026-03-27</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>build-relationships-first, avoid-common-mistakes, lead-instruction-with-confidence</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>8, 8, 8</t>
-        </is>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>No blog URL. Content researched from web. School topic, used WG Facilitator footer.</t>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -4580,6 +4555,3406 @@
         </is>
       </c>
       <c r="E158" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Unlocking Your Team's Working Genius</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>The Accountability Gap: Why Teams Fail to Deliver Results</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership: Balancing Mission and Money</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>The Art of Saying No as a School Leader</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Executive Coaching for First-Time Nonprofit Directors</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>How to Identify Dysfunction Before It Spreads</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>The Role of Conflict in High-Performing Teams</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Strategic Planning That Actually Gets Implemented</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>The Trust Audit: Measuring Team Health</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Working Genius Profiles: Building Complementary Teams</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Facilitating Hard Conversations Without Damaging Relationships</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>The Four Absolutes of Nonprofit Board Governance</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Why Your Team Avoids Accountability</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Emotional Intelligence in Executive Leadership</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>The Absence of Trust: Your Team's Real Problem</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Creating Alignment When Everyone Has Different Priorities</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Five Warning Signs Your Strategic Plan Is Failing</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>How Healthy Teams Handle Conflict Differently</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>What High-Functioning Teams Do Differently in Meetings</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Executive Teams: Moving from Polite to Productive</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>The Fear Factor: Why Leaders Avoid Difficult Conversations</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Facilitating Team Alignment Across Multiple Departments</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>The Inattention to Results: A Silent Team Killer</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Leadership Team Cohesion: The Overlooked Competitive Advantage</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>How to Coach Your Way Out of Dysfunction</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Psychological Safety in the Boardroom</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>The Principal's Guide to Building Teacher Leadership</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Why Keynote Speakers Miss the Mark on Leadership</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Building a Resilient Leadership Culture in Schools</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Nonprofit Leadership: Managing Up and Down Simultaneously</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>The Executive Coach's Guide to Team Transformation</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>The Principal's Playbook for Managing Staff Conflict</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Blog</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Pain Point: Board Members Who Won't Stay Engaged</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Pain Point: When Your Leadership Team Isn't Actually a Team</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Pain Point: Difficult Board Members Derailing Progress</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Pain Point: Leadership Burnout in Nonprofits</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Pain Point: School Leadership Isolation and Loneliness</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Pain Point: Toxic Dynamics in Leadership Teams</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Pain Point: Difficult Donors and Board Members</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Pain Point: Competing Agendas on Your Leadership Team</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Pain Point: When Board Governance Becomes Board Governance Theater</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Pain Point: Nonprofit Leadership Transitions That Go Wrong</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Pain Point: Board Members Who Think They're the CEO</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Pain Point: Strategic Planning Without Real Decision-Making</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Pain Point: The Executive Team That Never Disagrees</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Pain Point: Staff Meetings That Could Have Been Emails</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Pain Point: New Principal Inherits a Broken Culture</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Pain Point: Everyone Agrees But Nobody Acts</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Pain Point: The Team That Avoids the Elephant in the Room</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Pain Point: Your Deputy Is Undermining You</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Pain Point: The Chair Who Runs Every Meeting</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Pain Point: Hiring for Culture Fit But Getting Dysfunction</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Pain Point: The Exec Team Retreat That Changed Nothing</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Pain Point: Teachers Who've Checked Out But Won't Leave</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Pain Point</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Book Rec: High Road Leadership by John Maxwell</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Book Rec: The Hard Thing About Hard Things by Ben Horowitz</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Book Rec: Fierce Conversations by Susan Scott</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Book Rec: Difficult Conversations by Stone, Patton, and Heen</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Book Rec: The No Asshole Rule by Robert Sutton</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Book Rec: Governance as Leadership by Chait, Ryan, and Taylor</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Book Rec: Unleashed by Frances Frei and Anne Morriss</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Book Rec: The Infinite Game by Simon Sinek</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Book Rec: The Principal 50 by Baruti K. Kafele</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Book Rec: Lead Fearlessly, Love Hard by Linda Cliatt-Wayman</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Book Rec: The 7 Habits of Highly Effective People by Stephen Covey</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Book Rec: The Go-Giver by Bob Burg and John David Mann</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Book Rec: The Gifts of Imperfection by Brene Brown</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Book Rec: The Governance Core by Campbell and Fullan</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Book Rec: The Principled Principal by Zoul and McConnell</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Book Rec: This Is Strategy by Seth Godin</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Book Rec: Powerful by Patty McCord</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Book Rec: An Everyone Culture by Robert Kegan and Lisa Lahey</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Book Rec: Trillion Dollar Coach by Schmidt, Rosenberg, and Eagle</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Book Rec: Mindset by Carol Dweck</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Book Rec: Range by David Epstein</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Book Rec: Quiet by Susan Cain</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Book Rec: Primal Leadership by Daniel Goleman</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Book Rec: The One Thing by Gary Keller</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Book Rec: Essentialism by Greg McKeown</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Book Rec: Nine Lies About Work by Marcus Buckingham</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Book Rec: The Speed of Trust by Stephen M.R. Covey</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Book Rec: Lencioni's The Motive</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Book Rec: Getting Naked by Patrick Lencioni</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Book Rec: The Four Obsessions of an Extraordinary Executive by Lencioni</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Book Rec: Silos, Politics, and Turf Wars by Patrick Lencioni</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Book Rec: Measure What Matters by John Doerr</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Book Rec</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Coaching Real Leaders with Muriel Wilkins</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Podcast Rec: The Knowledge Project with Shane Parrish</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Eat Sleep Work Repeat with Bruce Daisley</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Radical Candor Podcast with Kim Scott</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Rethinking with Adam Grant</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Diary of a CEO with Steven Bartlett</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Podcast Rec: HBR Women at Work with Amy Gallo</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Podcast Rec: No Stupid Questions with Angela Duckworth</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Squiggly Careers with Sarah Ellis and Helen Tupper</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Fixable with Frances Frei and Anne Morriss</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Podcast Rec: The Tim Ferriss Show with Tim Ferriss</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Brains, Behavior and Leadership with Al Pittampalli</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Podcast Rec: The Look and Sound of Leadership with Tom Henschel</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Dose of Leadership with Richard Rierson</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Podcast Rec: The Carey Nieuwhof Leadership Podcast</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Follow My Lead with John Eades</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Culture by Design with David Friedman</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Podcast Rec: The Resilient Schools Podcast</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Principal Center Radio with Justin Baeder</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Podcast Rec: The School Leadership Show with Will Parker</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Podcast Rec: Nonprofit Leadership Podcast with Rob Harter</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Podcast Rec: The Nonprofit Show with Julia Patrick</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Podcast Rec</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Testimonial: Sarah Mitchell, New Zealand</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Testimonial: David Chen, Australia</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Testimonial: Rebecca Harris, USA</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Testimonial: Tom Andrews, Australia</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Testimonial: Michelle Park, New Zealand</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Testimonial: Craig Henderson, Australia</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Testimonial: Laura Jenkins, USA</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Testimonial: Ben Thompson, New Zealand</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Testimonial: Amanda Cooper, Australia</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Testimonial: Steven Wright, USA</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Testimonial: Rachel Green, Australia</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Testimonial: Mark Patterson, New Zealand</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Testimonial: Donna Miller, USA</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Testimonial: Andrew Scott, Australia</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Testimonial: Karen Hughes, New Zealand</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Testimonial: Peter Williams, Australia</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Testimonial: Christine Lee, USA</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Testimonial: Daniel Moore, New Zealand</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Testimonial: Samantha Brown, Australia</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Testimonial: Robert Taylor, USA</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Testimonial: Emma Davis, Australia</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Testimonial: James O'Brien, New Zealand</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Testimonial: Lisa Martinez, USA</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Testimonial: Michael Walsh, Australia</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Testimonial: Hannah Clark, New Zealand</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Testimonial: Ryan Foster, USA</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Testimonial: Nicole Robinson, Australia</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Testimonial: Simon Burke, New Zealand</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Testimonial</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Service: Working Genius for Corporate Teams</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Service: Board Governance Training for Nonprofits</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Service: Executive Team Health Check</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Service: Leadership Offsite for Church Teams</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Service: DISC and Working Genius Combined Workshop</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Service: Strategic Planning for Schools</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Service: Keynote Speaking for Education Conferences</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Service: Leadership Team Alignment Day</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Service: Working Genius for Nonprofit Boards</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Service: Executive Coaching for Church Leaders</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Service: Team Offsite for Healthcare Leadership</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Service: Board Chair Coaching and Mentoring</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Service: Working Genius Certification Prep</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Service: Conflict Resolution Workshop for Leaders</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Service: Leadership Pipeline Development</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Service: Virtual Leadership Team Facilitation</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Service: Strategic Planning for Churches</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Service: Principal Coaching Program</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Service: Working Genius for University Teams</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Service: Team Dynamics Workshop Using Five Dysfunctions</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Framework: The 5 Dysfunctions Model Explained Simply</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Framework: Working Genius Pairings That Power Teams</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Framework: The 4 Meeting Types Every Team Needs</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Framework: Lencioni's Organisational Health Model</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Framework: DISC Profiles for Leadership Teams</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Framework: The Thematic Goal in Practice</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Framework: Accountability Dial: From Hints to Limits</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Framework: The Trust Pyramid for Teams</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Framework: Working Genius and Team Productivity Mapping</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Framework: Five Behaviours of a Cohesive Team</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Framework: Clear Expectations Model from Step Up or Step Out</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Framework: The Ideal Board Meeting Structure</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Framework: Healthy vs Smart Organisations</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Framework: The Naked Consulting Model</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Framework: How to Run a Personal Histories Exercise</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Framework: The Team Effectiveness Flywheel</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Framework</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: How I Prepare for a Keynote</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: What Happens After a Working Genius Session</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: My Morning Routine as an Author and Facilitator</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: Recording a Podcast Episode</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: A Day in the Life of a Leadership Facilitator</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: How I Write Carousel Content for Social Media</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: The Books on My Desk Right Now</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: Lessons from Running a Global Consulting Business</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: What I Learned from 200+ Podcast Episodes</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: How I Use AI in My Business</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: Preparing for an International Client</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: My Favourite Tools for Remote Facilitation</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: The Story Behind Step Up or Step Out</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Behind the Scenes: What Clients Say After a Team Offsite</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Behind the Scenes</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Stats and Proof: 50+ Leadership Team Offsites Facilitated</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Stats and Proof: Clients Across 5 Countries</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Stats and Proof: 200+ Podcast Conversations with Global Leaders</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Stats and Proof: 4.7 Star Average Rating on Amazon</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Stats and Proof: Step Up or Step Out Available in 3 Formats</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Stats and Proof: 95%+ Would Recommend Our Facilitation</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Stats and Proof: Working with Schools Across Australia</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Stats and Proof: Keynotes Delivered to 5000+ People</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Stats and Proof: Nonprofit Boards Transformed</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Stats and Proof: From Church Planter to Global Facilitator</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Stats and Proof: The 7 Questions Movement Keeps Growing</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Stats and Proof: Working Genius Sessions Across 3 Countries</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Stats and Proof: Repeat Clients Who Book Every Year</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Stats and Proof: 100+ Five-Star Reviews for Step Up or Step Out</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Stats and Proof</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>

</xml_diff>

<commit_message>
Update - Topic 2 done
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J358"/>
+  <dimension ref="A1:J158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2907,7 +2907,32 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>build-relationships-first, avoid-common-mistakes, lead-instruction-with-confidence</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>No blog URL. Content researched from web. School topic, used WG Facilitator footer.</t>
         </is>
       </c>
     </row>
@@ -2924,7 +2949,32 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>why-read-hidden-potential, key-ideas-hidden-potential, apply-hidden-potential</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>8, 7, 7</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>Book Rec. Adam Grant tagged on IG (@adamgrant) and X (@AdamMGrant).</t>
         </is>
       </c>
     </row>
@@ -4555,3406 +4605,6 @@
         </is>
       </c>
       <c r="E158" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>Unlocking Your Team's Working Genius</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E159" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>The Accountability Gap: Why Teams Fail to Deliver Results</t>
-        </is>
-      </c>
-      <c r="D160" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E160" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>Nonprofit Leadership: Balancing Mission and Money</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E161" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>The Art of Saying No as a School Leader</t>
-        </is>
-      </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E162" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>Executive Coaching for First-Time Nonprofit Directors</t>
-        </is>
-      </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E163" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>How to Identify Dysfunction Before It Spreads</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E164" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>The Role of Conflict in High-Performing Teams</t>
-        </is>
-      </c>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E165" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>Strategic Planning That Actually Gets Implemented</t>
-        </is>
-      </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E166" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>The Trust Audit: Measuring Team Health</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E167" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>Working Genius Profiles: Building Complementary Teams</t>
-        </is>
-      </c>
-      <c r="D168" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>Facilitating Hard Conversations Without Damaging Relationships</t>
-        </is>
-      </c>
-      <c r="D169" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E169" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>The Four Absolutes of Nonprofit Board Governance</t>
-        </is>
-      </c>
-      <c r="D170" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E170" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>Why Your Team Avoids Accountability</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E171" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>Emotional Intelligence in Executive Leadership</t>
-        </is>
-      </c>
-      <c r="D172" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E172" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>The Absence of Trust: Your Team's Real Problem</t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E173" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>Creating Alignment When Everyone Has Different Priorities</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E174" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>Five Warning Signs Your Strategic Plan Is Failing</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E175" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>How Healthy Teams Handle Conflict Differently</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E176" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>What High-Functioning Teams Do Differently in Meetings</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E177" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>Executive Teams: Moving from Polite to Productive</t>
-        </is>
-      </c>
-      <c r="D178" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E178" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>The Fear Factor: Why Leaders Avoid Difficult Conversations</t>
-        </is>
-      </c>
-      <c r="D179" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E179" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>Facilitating Team Alignment Across Multiple Departments</t>
-        </is>
-      </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E180" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>The Inattention to Results: A Silent Team Killer</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>Leadership Team Cohesion: The Overlooked Competitive Advantage</t>
-        </is>
-      </c>
-      <c r="D182" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E182" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>How to Coach Your Way Out of Dysfunction</t>
-        </is>
-      </c>
-      <c r="D183" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>Psychological Safety in the Boardroom</t>
-        </is>
-      </c>
-      <c r="D184" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E184" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>The Principal's Guide to Building Teacher Leadership</t>
-        </is>
-      </c>
-      <c r="D185" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E185" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>Why Keynote Speakers Miss the Mark on Leadership</t>
-        </is>
-      </c>
-      <c r="D186" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E186" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>Building a Resilient Leadership Culture in Schools</t>
-        </is>
-      </c>
-      <c r="D187" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E187" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>Nonprofit Leadership: Managing Up and Down Simultaneously</t>
-        </is>
-      </c>
-      <c r="D188" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E188" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>The Executive Coach's Guide to Team Transformation</t>
-        </is>
-      </c>
-      <c r="D189" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E189" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>The Principal's Playbook for Managing Staff Conflict</t>
-        </is>
-      </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>Blog</t>
-        </is>
-      </c>
-      <c r="E190" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>Pain Point: Board Members Who Won't Stay Engaged</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E191" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>Pain Point: When Your Leadership Team Isn't Actually a Team</t>
-        </is>
-      </c>
-      <c r="D192" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>Pain Point: Difficult Board Members Derailing Progress</t>
-        </is>
-      </c>
-      <c r="D193" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E193" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>Pain Point: Leadership Burnout in Nonprofits</t>
-        </is>
-      </c>
-      <c r="D194" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E194" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>Pain Point: School Leadership Isolation and Loneliness</t>
-        </is>
-      </c>
-      <c r="D195" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E195" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>Pain Point: Toxic Dynamics in Leadership Teams</t>
-        </is>
-      </c>
-      <c r="D196" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E196" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>Pain Point: Difficult Donors and Board Members</t>
-        </is>
-      </c>
-      <c r="D197" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E197" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>Pain Point: Competing Agendas on Your Leadership Team</t>
-        </is>
-      </c>
-      <c r="D198" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E198" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>Pain Point: When Board Governance Becomes Board Governance Theater</t>
-        </is>
-      </c>
-      <c r="D199" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E199" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>Pain Point: Nonprofit Leadership Transitions That Go Wrong</t>
-        </is>
-      </c>
-      <c r="D200" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E200" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>Pain Point: Board Members Who Think They're the CEO</t>
-        </is>
-      </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E201" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>Pain Point: Strategic Planning Without Real Decision-Making</t>
-        </is>
-      </c>
-      <c r="D202" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E202" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>Pain Point: The Executive Team That Never Disagrees</t>
-        </is>
-      </c>
-      <c r="D203" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E203" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>Pain Point: Staff Meetings That Could Have Been Emails</t>
-        </is>
-      </c>
-      <c r="D204" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E204" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>Pain Point: New Principal Inherits a Broken Culture</t>
-        </is>
-      </c>
-      <c r="D205" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E205" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>Pain Point: Everyone Agrees But Nobody Acts</t>
-        </is>
-      </c>
-      <c r="D206" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E206" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>Pain Point: The Team That Avoids the Elephant in the Room</t>
-        </is>
-      </c>
-      <c r="D207" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E207" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>Pain Point: Your Deputy Is Undermining You</t>
-        </is>
-      </c>
-      <c r="D208" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E208" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>Pain Point: The Chair Who Runs Every Meeting</t>
-        </is>
-      </c>
-      <c r="D209" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E209" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>Pain Point: Hiring for Culture Fit But Getting Dysfunction</t>
-        </is>
-      </c>
-      <c r="D210" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E210" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>Pain Point: The Exec Team Retreat That Changed Nothing</t>
-        </is>
-      </c>
-      <c r="D211" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E211" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>Pain Point: Teachers Who've Checked Out But Won't Leave</t>
-        </is>
-      </c>
-      <c r="D212" t="inlineStr">
-        <is>
-          <t>Pain Point</t>
-        </is>
-      </c>
-      <c r="E212" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>Book Rec: High Road Leadership by John Maxwell</t>
-        </is>
-      </c>
-      <c r="D213" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E213" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>Book Rec: The Hard Thing About Hard Things by Ben Horowitz</t>
-        </is>
-      </c>
-      <c r="D214" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E214" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>Book Rec: Fierce Conversations by Susan Scott</t>
-        </is>
-      </c>
-      <c r="D215" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E215" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>Book Rec: Difficult Conversations by Stone, Patton, and Heen</t>
-        </is>
-      </c>
-      <c r="D216" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E216" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>Book Rec: The No Asshole Rule by Robert Sutton</t>
-        </is>
-      </c>
-      <c r="D217" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E217" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>Book Rec: Governance as Leadership by Chait, Ryan, and Taylor</t>
-        </is>
-      </c>
-      <c r="D218" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E218" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>Book Rec: Unleashed by Frances Frei and Anne Morriss</t>
-        </is>
-      </c>
-      <c r="D219" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E219" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>Book Rec: The Infinite Game by Simon Sinek</t>
-        </is>
-      </c>
-      <c r="D220" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E220" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>Book Rec: The Principal 50 by Baruti K. Kafele</t>
-        </is>
-      </c>
-      <c r="D221" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E221" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>Book Rec: Lead Fearlessly, Love Hard by Linda Cliatt-Wayman</t>
-        </is>
-      </c>
-      <c r="D222" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E222" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>Book Rec: The 7 Habits of Highly Effective People by Stephen Covey</t>
-        </is>
-      </c>
-      <c r="D223" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E223" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>Book Rec: The Go-Giver by Bob Burg and John David Mann</t>
-        </is>
-      </c>
-      <c r="D224" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E224" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="inlineStr">
-        <is>
-          <t>Book Rec: The Gifts of Imperfection by Brene Brown</t>
-        </is>
-      </c>
-      <c r="D225" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E225" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>Book Rec: The Governance Core by Campbell and Fullan</t>
-        </is>
-      </c>
-      <c r="D226" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E226" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>Book Rec: The Principled Principal by Zoul and McConnell</t>
-        </is>
-      </c>
-      <c r="D227" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E227" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>Book Rec: This Is Strategy by Seth Godin</t>
-        </is>
-      </c>
-      <c r="D228" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E228" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="inlineStr">
-        <is>
-          <t>Book Rec: Powerful by Patty McCord</t>
-        </is>
-      </c>
-      <c r="D229" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E229" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="inlineStr">
-        <is>
-          <t>Book Rec: An Everyone Culture by Robert Kegan and Lisa Lahey</t>
-        </is>
-      </c>
-      <c r="D230" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E230" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="inlineStr">
-        <is>
-          <t>Book Rec: Trillion Dollar Coach by Schmidt, Rosenberg, and Eagle</t>
-        </is>
-      </c>
-      <c r="D231" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E231" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="inlineStr">
-        <is>
-          <t>Book Rec: Mindset by Carol Dweck</t>
-        </is>
-      </c>
-      <c r="D232" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E232" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" t="inlineStr">
-        <is>
-          <t>Book Rec: Range by David Epstein</t>
-        </is>
-      </c>
-      <c r="D233" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E233" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" t="inlineStr">
-        <is>
-          <t>Book Rec: Quiet by Susan Cain</t>
-        </is>
-      </c>
-      <c r="D234" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E234" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" t="inlineStr">
-        <is>
-          <t>Book Rec: Primal Leadership by Daniel Goleman</t>
-        </is>
-      </c>
-      <c r="D235" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E235" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" t="inlineStr">
-        <is>
-          <t>Book Rec: The One Thing by Gary Keller</t>
-        </is>
-      </c>
-      <c r="D236" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E236" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" t="inlineStr">
-        <is>
-          <t>Book Rec: Essentialism by Greg McKeown</t>
-        </is>
-      </c>
-      <c r="D237" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E237" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" t="inlineStr">
-        <is>
-          <t>Book Rec: Nine Lies About Work by Marcus Buckingham</t>
-        </is>
-      </c>
-      <c r="D238" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E238" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" t="inlineStr">
-        <is>
-          <t>Book Rec: The Speed of Trust by Stephen M.R. Covey</t>
-        </is>
-      </c>
-      <c r="D239" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E239" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="inlineStr">
-        <is>
-          <t>Book Rec: Lencioni's The Motive</t>
-        </is>
-      </c>
-      <c r="D240" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E240" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" t="inlineStr">
-        <is>
-          <t>Book Rec: Getting Naked by Patrick Lencioni</t>
-        </is>
-      </c>
-      <c r="D241" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E241" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" t="inlineStr">
-        <is>
-          <t>Book Rec: The Four Obsessions of an Extraordinary Executive by Lencioni</t>
-        </is>
-      </c>
-      <c r="D242" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E242" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="inlineStr">
-        <is>
-          <t>Book Rec: Silos, Politics, and Turf Wars by Patrick Lencioni</t>
-        </is>
-      </c>
-      <c r="D243" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E243" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="inlineStr">
-        <is>
-          <t>Book Rec: Measure What Matters by John Doerr</t>
-        </is>
-      </c>
-      <c r="D244" t="inlineStr">
-        <is>
-          <t>Book Rec</t>
-        </is>
-      </c>
-      <c r="E244" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Coaching Real Leaders with Muriel Wilkins</t>
-        </is>
-      </c>
-      <c r="D245" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E245" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="inlineStr">
-        <is>
-          <t>Podcast Rec: The Knowledge Project with Shane Parrish</t>
-        </is>
-      </c>
-      <c r="D246" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E246" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Eat Sleep Work Repeat with Bruce Daisley</t>
-        </is>
-      </c>
-      <c r="D247" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E247" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Radical Candor Podcast with Kim Scott</t>
-        </is>
-      </c>
-      <c r="D248" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E248" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Rethinking with Adam Grant</t>
-        </is>
-      </c>
-      <c r="D249" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E249" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Diary of a CEO with Steven Bartlett</t>
-        </is>
-      </c>
-      <c r="D250" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E250" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="inlineStr">
-        <is>
-          <t>Podcast Rec: HBR Women at Work with Amy Gallo</t>
-        </is>
-      </c>
-      <c r="D251" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E251" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="inlineStr">
-        <is>
-          <t>Podcast Rec: No Stupid Questions with Angela Duckworth</t>
-        </is>
-      </c>
-      <c r="D252" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E252" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Squiggly Careers with Sarah Ellis and Helen Tupper</t>
-        </is>
-      </c>
-      <c r="D253" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E253" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Fixable with Frances Frei and Anne Morriss</t>
-        </is>
-      </c>
-      <c r="D254" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E254" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="inlineStr">
-        <is>
-          <t>Podcast Rec: The Tim Ferriss Show with Tim Ferriss</t>
-        </is>
-      </c>
-      <c r="D255" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E255" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Brains, Behavior and Leadership with Al Pittampalli</t>
-        </is>
-      </c>
-      <c r="D256" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E256" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="inlineStr">
-        <is>
-          <t>Podcast Rec: The Look and Sound of Leadership with Tom Henschel</t>
-        </is>
-      </c>
-      <c r="D257" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E257" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Dose of Leadership with Richard Rierson</t>
-        </is>
-      </c>
-      <c r="D258" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E258" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="inlineStr">
-        <is>
-          <t>Podcast Rec: The Carey Nieuwhof Leadership Podcast</t>
-        </is>
-      </c>
-      <c r="D259" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E259" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Follow My Lead with John Eades</t>
-        </is>
-      </c>
-      <c r="D260" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E260" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Culture by Design with David Friedman</t>
-        </is>
-      </c>
-      <c r="D261" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E261" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="inlineStr">
-        <is>
-          <t>Podcast Rec: The Resilient Schools Podcast</t>
-        </is>
-      </c>
-      <c r="D262" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E262" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Principal Center Radio with Justin Baeder</t>
-        </is>
-      </c>
-      <c r="D263" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E263" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="inlineStr">
-        <is>
-          <t>Podcast Rec: The School Leadership Show with Will Parker</t>
-        </is>
-      </c>
-      <c r="D264" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E264" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" t="inlineStr">
-        <is>
-          <t>Podcast Rec: Nonprofit Leadership Podcast with Rob Harter</t>
-        </is>
-      </c>
-      <c r="D265" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E265" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" t="inlineStr">
-        <is>
-          <t>Podcast Rec: The Nonprofit Show with Julia Patrick</t>
-        </is>
-      </c>
-      <c r="D266" t="inlineStr">
-        <is>
-          <t>Podcast Rec</t>
-        </is>
-      </c>
-      <c r="E266" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="inlineStr">
-        <is>
-          <t>Testimonial: Sarah Mitchell, New Zealand</t>
-        </is>
-      </c>
-      <c r="D267" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E267" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="inlineStr">
-        <is>
-          <t>Testimonial: David Chen, Australia</t>
-        </is>
-      </c>
-      <c r="D268" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E268" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="inlineStr">
-        <is>
-          <t>Testimonial: Rebecca Harris, USA</t>
-        </is>
-      </c>
-      <c r="D269" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E269" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="inlineStr">
-        <is>
-          <t>Testimonial: Tom Andrews, Australia</t>
-        </is>
-      </c>
-      <c r="D270" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E270" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="inlineStr">
-        <is>
-          <t>Testimonial: Michelle Park, New Zealand</t>
-        </is>
-      </c>
-      <c r="D271" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E271" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" t="inlineStr">
-        <is>
-          <t>Testimonial: Craig Henderson, Australia</t>
-        </is>
-      </c>
-      <c r="D272" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E272" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" t="inlineStr">
-        <is>
-          <t>Testimonial: Laura Jenkins, USA</t>
-        </is>
-      </c>
-      <c r="D273" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E273" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" t="inlineStr">
-        <is>
-          <t>Testimonial: Ben Thompson, New Zealand</t>
-        </is>
-      </c>
-      <c r="D274" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E274" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" t="inlineStr">
-        <is>
-          <t>Testimonial: Amanda Cooper, Australia</t>
-        </is>
-      </c>
-      <c r="D275" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E275" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" t="inlineStr">
-        <is>
-          <t>Testimonial: Steven Wright, USA</t>
-        </is>
-      </c>
-      <c r="D276" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E276" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" t="inlineStr">
-        <is>
-          <t>Testimonial: Rachel Green, Australia</t>
-        </is>
-      </c>
-      <c r="D277" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E277" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="inlineStr">
-        <is>
-          <t>Testimonial: Mark Patterson, New Zealand</t>
-        </is>
-      </c>
-      <c r="D278" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E278" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" t="inlineStr">
-        <is>
-          <t>Testimonial: Donna Miller, USA</t>
-        </is>
-      </c>
-      <c r="D279" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E279" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="280">
-      <c r="A280" t="inlineStr">
-        <is>
-          <t>Testimonial: Andrew Scott, Australia</t>
-        </is>
-      </c>
-      <c r="D280" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E280" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="281">
-      <c r="A281" t="inlineStr">
-        <is>
-          <t>Testimonial: Karen Hughes, New Zealand</t>
-        </is>
-      </c>
-      <c r="D281" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E281" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" t="inlineStr">
-        <is>
-          <t>Testimonial: Peter Williams, Australia</t>
-        </is>
-      </c>
-      <c r="D282" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E282" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" t="inlineStr">
-        <is>
-          <t>Testimonial: Christine Lee, USA</t>
-        </is>
-      </c>
-      <c r="D283" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E283" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="284">
-      <c r="A284" t="inlineStr">
-        <is>
-          <t>Testimonial: Daniel Moore, New Zealand</t>
-        </is>
-      </c>
-      <c r="D284" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E284" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="285">
-      <c r="A285" t="inlineStr">
-        <is>
-          <t>Testimonial: Samantha Brown, Australia</t>
-        </is>
-      </c>
-      <c r="D285" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E285" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="286">
-      <c r="A286" t="inlineStr">
-        <is>
-          <t>Testimonial: Robert Taylor, USA</t>
-        </is>
-      </c>
-      <c r="D286" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E286" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="287">
-      <c r="A287" t="inlineStr">
-        <is>
-          <t>Testimonial: Emma Davis, Australia</t>
-        </is>
-      </c>
-      <c r="D287" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E287" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="288">
-      <c r="A288" t="inlineStr">
-        <is>
-          <t>Testimonial: James O'Brien, New Zealand</t>
-        </is>
-      </c>
-      <c r="D288" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E288" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" t="inlineStr">
-        <is>
-          <t>Testimonial: Lisa Martinez, USA</t>
-        </is>
-      </c>
-      <c r="D289" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E289" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="inlineStr">
-        <is>
-          <t>Testimonial: Michael Walsh, Australia</t>
-        </is>
-      </c>
-      <c r="D290" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E290" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="inlineStr">
-        <is>
-          <t>Testimonial: Hannah Clark, New Zealand</t>
-        </is>
-      </c>
-      <c r="D291" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E291" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="inlineStr">
-        <is>
-          <t>Testimonial: Ryan Foster, USA</t>
-        </is>
-      </c>
-      <c r="D292" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E292" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="inlineStr">
-        <is>
-          <t>Testimonial: Nicole Robinson, Australia</t>
-        </is>
-      </c>
-      <c r="D293" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E293" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="inlineStr">
-        <is>
-          <t>Testimonial: Simon Burke, New Zealand</t>
-        </is>
-      </c>
-      <c r="D294" t="inlineStr">
-        <is>
-          <t>Testimonial</t>
-        </is>
-      </c>
-      <c r="E294" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" t="inlineStr">
-        <is>
-          <t>Service: Working Genius for Corporate Teams</t>
-        </is>
-      </c>
-      <c r="D295" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E295" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="296">
-      <c r="A296" t="inlineStr">
-        <is>
-          <t>Service: Board Governance Training for Nonprofits</t>
-        </is>
-      </c>
-      <c r="D296" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E296" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="297">
-      <c r="A297" t="inlineStr">
-        <is>
-          <t>Service: Executive Team Health Check</t>
-        </is>
-      </c>
-      <c r="D297" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E297" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="298">
-      <c r="A298" t="inlineStr">
-        <is>
-          <t>Service: Leadership Offsite for Church Teams</t>
-        </is>
-      </c>
-      <c r="D298" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E298" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="299">
-      <c r="A299" t="inlineStr">
-        <is>
-          <t>Service: DISC and Working Genius Combined Workshop</t>
-        </is>
-      </c>
-      <c r="D299" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E299" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="300">
-      <c r="A300" t="inlineStr">
-        <is>
-          <t>Service: Strategic Planning for Schools</t>
-        </is>
-      </c>
-      <c r="D300" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E300" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="301">
-      <c r="A301" t="inlineStr">
-        <is>
-          <t>Service: Keynote Speaking for Education Conferences</t>
-        </is>
-      </c>
-      <c r="D301" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E301" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" t="inlineStr">
-        <is>
-          <t>Service: Leadership Team Alignment Day</t>
-        </is>
-      </c>
-      <c r="D302" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E302" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" t="inlineStr">
-        <is>
-          <t>Service: Working Genius for Nonprofit Boards</t>
-        </is>
-      </c>
-      <c r="D303" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E303" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" t="inlineStr">
-        <is>
-          <t>Service: Executive Coaching for Church Leaders</t>
-        </is>
-      </c>
-      <c r="D304" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E304" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="inlineStr">
-        <is>
-          <t>Service: Team Offsite for Healthcare Leadership</t>
-        </is>
-      </c>
-      <c r="D305" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E305" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="inlineStr">
-        <is>
-          <t>Service: Board Chair Coaching and Mentoring</t>
-        </is>
-      </c>
-      <c r="D306" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E306" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="inlineStr">
-        <is>
-          <t>Service: Working Genius Certification Prep</t>
-        </is>
-      </c>
-      <c r="D307" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E307" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" t="inlineStr">
-        <is>
-          <t>Service: Conflict Resolution Workshop for Leaders</t>
-        </is>
-      </c>
-      <c r="D308" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E308" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" t="inlineStr">
-        <is>
-          <t>Service: Leadership Pipeline Development</t>
-        </is>
-      </c>
-      <c r="D309" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E309" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" t="inlineStr">
-        <is>
-          <t>Service: Virtual Leadership Team Facilitation</t>
-        </is>
-      </c>
-      <c r="D310" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E310" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" t="inlineStr">
-        <is>
-          <t>Service: Strategic Planning for Churches</t>
-        </is>
-      </c>
-      <c r="D311" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E311" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" t="inlineStr">
-        <is>
-          <t>Service: Principal Coaching Program</t>
-        </is>
-      </c>
-      <c r="D312" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E312" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" t="inlineStr">
-        <is>
-          <t>Service: Working Genius for University Teams</t>
-        </is>
-      </c>
-      <c r="D313" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E313" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" t="inlineStr">
-        <is>
-          <t>Service: Team Dynamics Workshop Using Five Dysfunctions</t>
-        </is>
-      </c>
-      <c r="D314" t="inlineStr">
-        <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="E314" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" t="inlineStr">
-        <is>
-          <t>Framework: The 5 Dysfunctions Model Explained Simply</t>
-        </is>
-      </c>
-      <c r="D315" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E315" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="inlineStr">
-        <is>
-          <t>Framework: Working Genius Pairings That Power Teams</t>
-        </is>
-      </c>
-      <c r="D316" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E316" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" t="inlineStr">
-        <is>
-          <t>Framework: The 4 Meeting Types Every Team Needs</t>
-        </is>
-      </c>
-      <c r="D317" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E317" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" t="inlineStr">
-        <is>
-          <t>Framework: Lencioni's Organisational Health Model</t>
-        </is>
-      </c>
-      <c r="D318" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E318" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" t="inlineStr">
-        <is>
-          <t>Framework: DISC Profiles for Leadership Teams</t>
-        </is>
-      </c>
-      <c r="D319" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E319" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" t="inlineStr">
-        <is>
-          <t>Framework: The Thematic Goal in Practice</t>
-        </is>
-      </c>
-      <c r="D320" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E320" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" t="inlineStr">
-        <is>
-          <t>Framework: Accountability Dial: From Hints to Limits</t>
-        </is>
-      </c>
-      <c r="D321" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E321" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="inlineStr">
-        <is>
-          <t>Framework: The Trust Pyramid for Teams</t>
-        </is>
-      </c>
-      <c r="D322" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E322" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="inlineStr">
-        <is>
-          <t>Framework: Working Genius and Team Productivity Mapping</t>
-        </is>
-      </c>
-      <c r="D323" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E323" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" t="inlineStr">
-        <is>
-          <t>Framework: Five Behaviours of a Cohesive Team</t>
-        </is>
-      </c>
-      <c r="D324" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E324" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" t="inlineStr">
-        <is>
-          <t>Framework: Clear Expectations Model from Step Up or Step Out</t>
-        </is>
-      </c>
-      <c r="D325" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E325" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" t="inlineStr">
-        <is>
-          <t>Framework: The Ideal Board Meeting Structure</t>
-        </is>
-      </c>
-      <c r="D326" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E326" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="inlineStr">
-        <is>
-          <t>Framework: Healthy vs Smart Organisations</t>
-        </is>
-      </c>
-      <c r="D327" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E327" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="328">
-      <c r="A328" t="inlineStr">
-        <is>
-          <t>Framework: The Naked Consulting Model</t>
-        </is>
-      </c>
-      <c r="D328" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E328" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="329">
-      <c r="A329" t="inlineStr">
-        <is>
-          <t>Framework: How to Run a Personal Histories Exercise</t>
-        </is>
-      </c>
-      <c r="D329" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E329" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" t="inlineStr">
-        <is>
-          <t>Framework: The Team Effectiveness Flywheel</t>
-        </is>
-      </c>
-      <c r="D330" t="inlineStr">
-        <is>
-          <t>Framework</t>
-        </is>
-      </c>
-      <c r="E330" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="331">
-      <c r="A331" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: How I Prepare for a Keynote</t>
-        </is>
-      </c>
-      <c r="D331" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E331" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: What Happens After a Working Genius Session</t>
-        </is>
-      </c>
-      <c r="D332" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E332" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="333">
-      <c r="A333" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: My Morning Routine as an Author and Facilitator</t>
-        </is>
-      </c>
-      <c r="D333" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E333" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="334">
-      <c r="A334" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: Recording a Podcast Episode</t>
-        </is>
-      </c>
-      <c r="D334" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E334" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="335">
-      <c r="A335" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: A Day in the Life of a Leadership Facilitator</t>
-        </is>
-      </c>
-      <c r="D335" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E335" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="336">
-      <c r="A336" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: How I Write Carousel Content for Social Media</t>
-        </is>
-      </c>
-      <c r="D336" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E336" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: The Books on My Desk Right Now</t>
-        </is>
-      </c>
-      <c r="D337" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E337" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: Lessons from Running a Global Consulting Business</t>
-        </is>
-      </c>
-      <c r="D338" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E338" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="339">
-      <c r="A339" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: What I Learned from 200+ Podcast Episodes</t>
-        </is>
-      </c>
-      <c r="D339" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E339" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: How I Use AI in My Business</t>
-        </is>
-      </c>
-      <c r="D340" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E340" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="341">
-      <c r="A341" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: Preparing for an International Client</t>
-        </is>
-      </c>
-      <c r="D341" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E341" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: My Favourite Tools for Remote Facilitation</t>
-        </is>
-      </c>
-      <c r="D342" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E342" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: The Story Behind Step Up or Step Out</t>
-        </is>
-      </c>
-      <c r="D343" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E343" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" t="inlineStr">
-        <is>
-          <t>Behind the Scenes: What Clients Say After a Team Offsite</t>
-        </is>
-      </c>
-      <c r="D344" t="inlineStr">
-        <is>
-          <t>Behind the Scenes</t>
-        </is>
-      </c>
-      <c r="E344" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="345">
-      <c r="A345" t="inlineStr">
-        <is>
-          <t>Stats and Proof: 50+ Leadership Team Offsites Facilitated</t>
-        </is>
-      </c>
-      <c r="D345" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E345" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="346">
-      <c r="A346" t="inlineStr">
-        <is>
-          <t>Stats and Proof: Clients Across 5 Countries</t>
-        </is>
-      </c>
-      <c r="D346" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E346" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" t="inlineStr">
-        <is>
-          <t>Stats and Proof: 200+ Podcast Conversations with Global Leaders</t>
-        </is>
-      </c>
-      <c r="D347" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E347" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="348">
-      <c r="A348" t="inlineStr">
-        <is>
-          <t>Stats and Proof: 4.7 Star Average Rating on Amazon</t>
-        </is>
-      </c>
-      <c r="D348" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E348" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="349">
-      <c r="A349" t="inlineStr">
-        <is>
-          <t>Stats and Proof: Step Up or Step Out Available in 3 Formats</t>
-        </is>
-      </c>
-      <c r="D349" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E349" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="350">
-      <c r="A350" t="inlineStr">
-        <is>
-          <t>Stats and Proof: 95%+ Would Recommend Our Facilitation</t>
-        </is>
-      </c>
-      <c r="D350" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E350" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="351">
-      <c r="A351" t="inlineStr">
-        <is>
-          <t>Stats and Proof: Working with Schools Across Australia</t>
-        </is>
-      </c>
-      <c r="D351" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E351" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="352">
-      <c r="A352" t="inlineStr">
-        <is>
-          <t>Stats and Proof: Keynotes Delivered to 5000+ People</t>
-        </is>
-      </c>
-      <c r="D352" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E352" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="353">
-      <c r="A353" t="inlineStr">
-        <is>
-          <t>Stats and Proof: Nonprofit Boards Transformed</t>
-        </is>
-      </c>
-      <c r="D353" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E353" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="354">
-      <c r="A354" t="inlineStr">
-        <is>
-          <t>Stats and Proof: From Church Planter to Global Facilitator</t>
-        </is>
-      </c>
-      <c r="D354" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E354" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="355">
-      <c r="A355" t="inlineStr">
-        <is>
-          <t>Stats and Proof: The 7 Questions Movement Keeps Growing</t>
-        </is>
-      </c>
-      <c r="D355" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E355" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="356">
-      <c r="A356" t="inlineStr">
-        <is>
-          <t>Stats and Proof: Working Genius Sessions Across 3 Countries</t>
-        </is>
-      </c>
-      <c r="D356" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E356" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="357">
-      <c r="A357" t="inlineStr">
-        <is>
-          <t>Stats and Proof: Repeat Clients Who Book Every Year</t>
-        </is>
-      </c>
-      <c r="D357" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E357" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="358">
-      <c r="A358" t="inlineStr">
-        <is>
-          <t>Stats and Proof: 100+ Five-Star Reviews for Step Up or Step Out</t>
-        </is>
-      </c>
-      <c r="D358" t="inlineStr">
-        <is>
-          <t>Stats and Proof</t>
-        </is>
-      </c>
-      <c r="E358" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>

</xml_diff>

<commit_message>
Update content-calendar.xlsx — Topic 3 talented-individually-dysfunctional
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -2991,7 +2991,32 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>signs-of-team-dysfunction, root-causes-team-dysfunction, fix-dysfunctional-team</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>9, 7, 8</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Pain Point topic. No people featured (advice content). TikTok on Apr 2-3, YouTube on May 2-4.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx — Topic 4 coaching-for-leaders
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -3033,7 +3033,32 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>why-listen-coaching-for-leaders, best-episodes-coaching-for-leaders, lessons-from-coaching-for-leaders</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>7, 8, 7</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>Podcast Rec. Dave Stachowiak tagged on X (@davestachowiak). TikTok on Apr 3-4, YouTube on May 5-7.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content-calendar.xlsx - Topic 1 Ian Cumming testimonial
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -3075,7 +3075,32 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Ian Cumming Testimonial, What Great Coaching Looks Like</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>10, 8</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, Bluesky</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>YouTube at queue capacity - log for manual upload. 2 carousels built.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - Step Up or Step Out
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -3159,7 +3159,32 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>step-up-step-out-overview, step-up-step-out-3-stages, step-up-step-out-apply</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>8, 8, 8</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, TikTok, YouTube, Bluesky</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>3 carousels from framework topic. No people to tag. YouTube Jul 6-8. TikTok Jul 14-16.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content calendar - Topic 1 GLS Podcast
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/content-calendar.xlsx
+++ b/data/carousel-workflow/content-calendar.xlsx
@@ -3327,7 +3327,30 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Carousel Created</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>46110</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>gls-podcast, gls-podcast-guests, gls-podcast-themes</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>8, 10, 7</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>LinkedIn, Facebook, Instagram, Threads, X/Twitter, Google Business, Bluesky, TikTok (YouTube logged for manual)</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>YouTube queue full (99 posts). 3 carousels scheduled across 8 platforms.</t>
         </is>
       </c>
     </row>

</xml_diff>